<commit_message>
created TerritoryRequest.java class and added some attributes
</commit_message>
<xml_diff>
--- a/DWM.xlsx
+++ b/DWM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30215"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bnagritech1-my.sharepoint.com/personal/it_intern_bngroupindia_com/Documents/tradesphere/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="323" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{098DA5F3-A63C-48E1-BE73-F5470625A2FE}"/>
+  <xr:revisionPtr revIDLastSave="399" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8317B7A6-5347-40B4-8672-8C5CE52D8653}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DWM" sheetId="4" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="71">
   <si>
     <t>Pilot : Tradesphere</t>
   </si>
@@ -70,6 +70,9 @@
     <t>Status</t>
   </si>
   <si>
+    <t>weekend off included</t>
+  </si>
+  <si>
     <t>Phase 1</t>
   </si>
   <si>
@@ -79,19 +82,25 @@
     <t>Completed</t>
   </si>
   <si>
+    <t>Yes</t>
+  </si>
+  <si>
     <t>Phase 2</t>
   </si>
   <si>
+    <t>Database Design &amp; Architecture Setup</t>
+  </si>
+  <si>
+    <t>In-progress</t>
+  </si>
+  <si>
     <t>Not Started</t>
   </si>
   <si>
     <t>Phase 3</t>
   </si>
   <si>
-    <t>Database Design &amp; Architecture Setup</t>
-  </si>
-  <si>
-    <t>In-progress</t>
+    <t>Authentication Module</t>
   </si>
   <si>
     <t>In-Progress</t>
@@ -100,45 +109,102 @@
     <t>Phase 4</t>
   </si>
   <si>
+    <t>Security Module</t>
+  </si>
+  <si>
     <t>Phase 5</t>
   </si>
   <si>
+    <t>Employee Module</t>
+  </si>
+  <si>
     <t>Phase 6</t>
   </si>
   <si>
+    <t>Territory Module</t>
+  </si>
+  <si>
     <t>Phase 7</t>
   </si>
   <si>
+    <t>Promoter Module</t>
+  </si>
+  <si>
     <t>Phase 8</t>
   </si>
   <si>
+    <t>Beats &amp; Beat Assignment Module</t>
+  </si>
+  <si>
     <t>Phase 9</t>
   </si>
   <si>
+    <t>Retailer Module</t>
+  </si>
+  <si>
     <t>Phase 10</t>
   </si>
   <si>
+    <t>Attendance And EOD Module</t>
+  </si>
+  <si>
     <t>Phase 11</t>
   </si>
   <si>
+    <t>Visit Module</t>
+  </si>
+  <si>
     <t>Phase 12</t>
   </si>
   <si>
+    <t>Retailer Feedback Module</t>
+  </si>
+  <si>
     <t>Phase 13</t>
   </si>
   <si>
+    <t>Product Module</t>
+  </si>
+  <si>
     <t>Phase 14</t>
   </si>
   <si>
+    <t>Retailer Stock Management</t>
+  </si>
+  <si>
     <t>Phase 15</t>
   </si>
   <si>
+    <t>Order Module</t>
+  </si>
+  <si>
     <t>Phase 16</t>
   </si>
   <si>
+    <t>UI/UX Design(Portal + App)</t>
+  </si>
+  <si>
     <t>Phase 17</t>
   </si>
   <si>
+    <t>Dashboard &amp; Reporting</t>
+  </si>
+  <si>
+    <t>Phase 18</t>
+  </si>
+  <si>
+    <t>Testing, Bug fixing</t>
+  </si>
+  <si>
+    <t>Phase 19</t>
+  </si>
+  <si>
+    <t>Deployment And Go-live Suppot</t>
+  </si>
+  <si>
+    <t>Final Date</t>
+  </si>
+  <si>
     <t>Dependency (Task ID)</t>
   </si>
   <si>
@@ -185,66 +251,6 @@
   </si>
   <si>
     <t>Production Deployment</t>
-  </si>
-  <si>
-    <t>Beats &amp; Beat Assignment Module</t>
-  </si>
-  <si>
-    <t>Authentication Module</t>
-  </si>
-  <si>
-    <t>Security Module</t>
-  </si>
-  <si>
-    <t>Employee Module</t>
-  </si>
-  <si>
-    <t>Territory Module</t>
-  </si>
-  <si>
-    <t>Promoter Module</t>
-  </si>
-  <si>
-    <t>Retailer Module</t>
-  </si>
-  <si>
-    <t>Attendance And EOD Module</t>
-  </si>
-  <si>
-    <t>Visit Module</t>
-  </si>
-  <si>
-    <t>Product Module</t>
-  </si>
-  <si>
-    <t>Retailer Stock Management</t>
-  </si>
-  <si>
-    <t>Order Module</t>
-  </si>
-  <si>
-    <t>UI/UX Design(Portal + App)</t>
-  </si>
-  <si>
-    <t>Dashboard &amp; Reporting</t>
-  </si>
-  <si>
-    <t>Phase 18</t>
-  </si>
-  <si>
-    <t>Testing, Bug fixing</t>
-  </si>
-  <si>
-    <t>Phase 19</t>
-  </si>
-  <si>
-    <t>Deployment And Go-live Suppot</t>
-  </si>
-  <si>
-    <t>Retailer Feedback Module</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Final date :- 31-Oct-26</t>
   </si>
 </sst>
 </file>
@@ -255,7 +261,7 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
     <numFmt numFmtId="165" formatCode="[$-409]dd\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -277,15 +283,21 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -332,11 +344,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -353,12 +378,21 @@
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -405,10 +439,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -675,137 +705,137 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A0EB679-3C26-4760-A69A-4B3B2033083D}">
   <dimension ref="A1:A34"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1">
       <c r="A2" s="6">
         <v>46174</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1">
       <c r="A3" s="6">
         <v>46175</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1">
       <c r="A4" s="6">
         <v>46176</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1">
       <c r="A5" s="6">
         <v>46177</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1">
       <c r="A6" s="6">
         <v>46178</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1">
       <c r="A7" s="6">
         <v>46179</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1">
       <c r="A8" s="6">
         <v>46180</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1">
       <c r="A9" s="6">
         <v>46181</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1">
       <c r="A10" s="6">
         <v>46182</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1">
       <c r="A11" s="6">
         <v>46183</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1">
       <c r="A12" s="6">
         <v>46184</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1">
       <c r="A13" s="6">
         <v>46185</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1">
       <c r="A14" s="6"/>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1">
       <c r="A15" s="6"/>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1">
       <c r="A16" s="6"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1">
       <c r="A17" s="6"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1">
       <c r="A18" s="6"/>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1">
       <c r="A19" s="6"/>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1">
       <c r="A20" s="6"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1">
       <c r="A21" s="6"/>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1">
       <c r="A22" s="6"/>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1">
       <c r="A23" s="6"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1">
       <c r="A24" s="6"/>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1">
       <c r="A25" s="6"/>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1">
       <c r="A26" s="6"/>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1">
       <c r="A27" s="6"/>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1">
       <c r="A28" s="6"/>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1">
       <c r="A29" s="6"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1">
       <c r="A30" s="6"/>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:1">
       <c r="A31" s="6"/>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:1">
       <c r="A32" s="6"/>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:1">
       <c r="A33" s="6"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:1">
       <c r="A34" s="6"/>
     </row>
   </sheetData>
@@ -816,18 +846,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45"/>
   <cols>
-    <col min="2" max="2" width="14.453125" customWidth="1"/>
-    <col min="3" max="3" width="41.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.26953125" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="3" max="3" width="41.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="7" max="8" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.1796875" hidden="1" customWidth="1"/>
+    <col min="7" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.140625" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16">
       <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
@@ -836,7 +867,7 @@
       <c r="E1" s="11"/>
       <c r="F1" s="11"/>
     </row>
-    <row r="2" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="30.75">
       <c r="A2" s="7" t="s">
         <v>2</v>
       </c>
@@ -855,557 +886,619 @@
       <c r="F2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="15" t="s">
         <v>8</v>
       </c>
       <c r="H2" s="7" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I2" s="13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16">
       <c r="A3" s="3">
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="3">
-        <v>1</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="D3" s="3"/>
       <c r="E3" s="9">
         <v>46181</v>
       </c>
       <c r="F3" s="3">
-        <v>7</v>
-      </c>
-      <c r="G3" s="10">
+        <v>9</v>
+      </c>
+      <c r="G3" s="16">
         <f>E3+F3</f>
-        <v>46188</v>
+        <v>46190</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="I3" s="14" t="s">
+        <v>14</v>
       </c>
       <c r="J3" s="2"/>
       <c r="P3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16">
       <c r="A4" s="3">
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="9">
         <f>G3+1</f>
-        <v>46189</v>
+        <v>46191</v>
       </c>
       <c r="F4" s="3">
-        <v>14</v>
-      </c>
-      <c r="G4" s="10">
+        <v>18</v>
+      </c>
+      <c r="G4" s="16">
         <f t="shared" ref="G4:G21" si="0">E4+F4</f>
-        <v>46203</v>
+        <v>46209</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>17</v>
       </c>
+      <c r="I4" s="14" t="s">
+        <v>14</v>
+      </c>
       <c r="P4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16">
       <c r="A5" s="3">
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="D5" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" s="9">
         <f>G4+1</f>
-        <v>46204</v>
+        <v>46210</v>
       </c>
       <c r="F5" s="3">
-        <v>5</v>
-      </c>
-      <c r="G5" s="10">
+        <v>7</v>
+      </c>
+      <c r="G5" s="16">
         <f t="shared" si="0"/>
-        <v>46209</v>
+        <v>46217</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>14</v>
       </c>
       <c r="P5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
       <c r="A6" s="3">
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="D6" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E6" s="9">
-        <f t="shared" ref="E6:E20" si="1">G5+1</f>
-        <v>46210</v>
+        <f t="shared" ref="E6:E19" si="1">G5+1</f>
+        <v>46218</v>
       </c>
       <c r="F6" s="3">
-        <v>5</v>
-      </c>
-      <c r="G6" s="10">
+        <v>2</v>
+      </c>
+      <c r="G6" s="16">
         <f t="shared" si="0"/>
-        <v>46215</v>
+        <v>46220</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="I6" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16">
       <c r="A7" s="3">
         <v>5</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="D7" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E7" s="9">
         <f t="shared" si="1"/>
-        <v>46216</v>
+        <v>46221</v>
       </c>
       <c r="F7" s="3">
-        <v>5</v>
-      </c>
-      <c r="G7" s="10">
+        <v>7</v>
+      </c>
+      <c r="G7" s="16">
         <f t="shared" si="0"/>
-        <v>46221</v>
+        <v>46228</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16">
       <c r="A8" s="3">
         <v>6</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="D8" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E8" s="9">
         <f t="shared" si="1"/>
-        <v>46222</v>
+        <v>46229</v>
       </c>
       <c r="F8" s="3">
-        <v>5</v>
-      </c>
-      <c r="G8" s="10">
+        <v>7</v>
+      </c>
+      <c r="G8" s="16">
         <f t="shared" si="0"/>
-        <v>46227</v>
+        <v>46236</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16">
       <c r="A9" s="3">
         <v>7</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="D9" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E9" s="9">
         <f t="shared" si="1"/>
-        <v>46228</v>
+        <v>46237</v>
       </c>
       <c r="F9" s="3">
-        <v>5</v>
-      </c>
-      <c r="G9" s="10">
+        <v>7</v>
+      </c>
+      <c r="G9" s="16">
         <f t="shared" si="0"/>
-        <v>46233</v>
+        <v>46244</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16">
       <c r="A10" s="3">
         <v>8</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="D10" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E10" s="9">
         <f t="shared" si="1"/>
-        <v>46234</v>
+        <v>46245</v>
       </c>
       <c r="F10" s="3">
-        <v>8</v>
-      </c>
-      <c r="G10" s="10">
+        <v>10</v>
+      </c>
+      <c r="G10" s="16">
         <f t="shared" si="0"/>
-        <v>46242</v>
+        <v>46255</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16">
       <c r="A11" s="3">
         <v>9</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="D11" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E11" s="9">
         <f t="shared" si="1"/>
-        <v>46243</v>
+        <v>46256</v>
       </c>
       <c r="F11" s="3">
-        <v>5</v>
-      </c>
-      <c r="G11" s="10">
+        <v>7</v>
+      </c>
+      <c r="G11" s="16">
         <f t="shared" si="0"/>
-        <v>46248</v>
+        <v>46263</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16">
       <c r="A12" s="3">
         <v>10</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="D12" s="3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E12" s="9">
         <f t="shared" si="1"/>
-        <v>46249</v>
+        <v>46264</v>
       </c>
       <c r="F12" s="3">
-        <v>7</v>
-      </c>
-      <c r="G12" s="10">
+        <v>9</v>
+      </c>
+      <c r="G12" s="16">
         <f t="shared" si="0"/>
-        <v>46256</v>
+        <v>46273</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16">
       <c r="A13" s="3">
         <v>11</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="D13" s="3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E13" s="9">
         <f t="shared" si="1"/>
-        <v>46257</v>
+        <v>46274</v>
       </c>
       <c r="F13" s="3">
-        <v>7</v>
-      </c>
-      <c r="G13" s="10">
+        <v>9</v>
+      </c>
+      <c r="G13" s="16">
         <f t="shared" si="0"/>
-        <v>46264</v>
+        <v>46283</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16">
       <c r="A14" s="3">
         <v>12</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="D14" s="3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E14" s="9">
         <f t="shared" si="1"/>
-        <v>46265</v>
+        <v>46284</v>
       </c>
       <c r="F14" s="3">
-        <v>3</v>
-      </c>
-      <c r="G14" s="10">
+        <v>5</v>
+      </c>
+      <c r="G14" s="16">
         <f t="shared" si="0"/>
-        <v>46268</v>
+        <v>46289</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16">
       <c r="A15" s="3">
         <v>13</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="D15" s="3">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E15" s="9">
         <f t="shared" si="1"/>
-        <v>46269</v>
+        <v>46290</v>
       </c>
       <c r="F15" s="3">
-        <v>3</v>
-      </c>
-      <c r="G15" s="10">
+        <v>5</v>
+      </c>
+      <c r="G15" s="16">
         <f t="shared" si="0"/>
-        <v>46272</v>
+        <v>46295</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16">
       <c r="A16" s="3">
         <v>14</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="D16" s="3">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E16" s="9">
         <f t="shared" si="1"/>
-        <v>46273</v>
+        <v>46296</v>
       </c>
       <c r="F16" s="3">
-        <v>7</v>
-      </c>
-      <c r="G16" s="10">
+        <v>9</v>
+      </c>
+      <c r="G16" s="16">
         <f t="shared" si="0"/>
-        <v>46280</v>
+        <v>46305</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" s="3">
         <v>15</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="D17" s="3">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E17" s="9">
         <f t="shared" si="1"/>
-        <v>46281</v>
+        <v>46306</v>
       </c>
       <c r="F17" s="3">
-        <v>5</v>
-      </c>
-      <c r="G17" s="10">
+        <v>7</v>
+      </c>
+      <c r="G17" s="16">
         <f t="shared" si="0"/>
-        <v>46286</v>
+        <v>46313</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
       <c r="A18" s="3">
         <v>16</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="D18" s="3">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E18" s="9">
         <f t="shared" si="1"/>
-        <v>46287</v>
+        <v>46314</v>
       </c>
       <c r="F18" s="3">
-        <v>15</v>
-      </c>
-      <c r="G18" s="10">
+        <v>19</v>
+      </c>
+      <c r="G18" s="16">
         <f t="shared" si="0"/>
-        <v>46302</v>
+        <v>46333</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I18" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
       <c r="A19" s="3">
         <v>17</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="D19" s="3">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E19" s="9">
         <f t="shared" si="1"/>
-        <v>46303</v>
+        <v>46334</v>
       </c>
       <c r="F19" s="3">
-        <v>7</v>
-      </c>
-      <c r="G19" s="10">
+        <v>9</v>
+      </c>
+      <c r="G19" s="16">
         <f t="shared" si="0"/>
-        <v>46310</v>
+        <v>46343</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I19" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" s="3">
         <v>18</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>64</v>
+        <v>50</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>51</v>
       </c>
       <c r="D20" s="3">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E20" s="9">
         <f>G19+1</f>
-        <v>46311</v>
+        <v>46344</v>
       </c>
       <c r="F20" s="3">
-        <v>7</v>
-      </c>
-      <c r="G20" s="10">
+        <v>9</v>
+      </c>
+      <c r="G20" s="16">
         <f t="shared" si="0"/>
-        <v>46318</v>
+        <v>46353</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="I20" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
       <c r="A21" s="3">
         <v>19</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="D21" s="3">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E21" s="9">
         <f>G20+1</f>
-        <v>46319</v>
+        <v>46354</v>
       </c>
       <c r="F21" s="3">
-        <v>7</v>
-      </c>
-      <c r="G21" s="10">
+        <v>9</v>
+      </c>
+      <c r="G21" s="16">
         <f t="shared" si="0"/>
-        <v>46326</v>
-      </c>
-      <c r="H21" s="13" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+        <v>46363</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="15">
       <c r="C23" s="3" t="s">
-        <v>68</v>
+        <v>54</v>
+      </c>
+      <c r="D23" s="12">
+        <f>G21</f>
+        <v>46363</v>
       </c>
     </row>
   </sheetData>
@@ -1413,13 +1506,13 @@
     <mergeCell ref="B1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="H3:H21">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="7" operator="equal">
       <formula>$P$5</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="8" operator="equal">
       <formula>$P$3</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="9" operator="equal">
       <formula>$P$4</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1430,9 +1523,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBB1C660-FD22-424D-B761-DA960EAAB43D}">
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -1443,7 +1536,7 @@
         <v>4</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>6</v>
@@ -1458,35 +1551,35 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>57</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="F2">
         <v>2</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1495,15 +1588,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>61</v>
       </c>
       <c r="D4">
         <v>2</v>
@@ -1512,15 +1605,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>63</v>
       </c>
       <c r="D5">
         <v>3</v>
@@ -1529,15 +1622,15 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="C6" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="D6">
         <v>4</v>
@@ -1546,15 +1639,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>66</v>
       </c>
       <c r="D7">
         <v>5</v>
@@ -1563,15 +1656,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>68</v>
       </c>
       <c r="D8">
         <v>6</v>
@@ -1580,15 +1673,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="D9">
         <v>7</v>

</xml_diff>

<commit_message>
Created ResourceNotFoundException.java exception class
</commit_message>
<xml_diff>
--- a/DWM.xlsx
+++ b/DWM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bnagritech1-my.sharepoint.com/personal/it_intern_bngroupindia_com/Documents/tradesphere/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="399" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8317B7A6-5347-40B4-8672-8C5CE52D8653}"/>
+  <xr:revisionPtr revIDLastSave="400" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25B65384-2C40-4578-ADFB-AC7F8B49A189}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1140" yWindow="1140" windowWidth="14400" windowHeight="7270" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DWM" sheetId="4" r:id="rId1"/>
@@ -261,7 +261,7 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
     <numFmt numFmtId="165" formatCode="[$-409]dd\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -379,9 +379,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -393,6 +390,9 @@
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -705,137 +705,137 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A0EB679-3C26-4760-A69A-4B3B2033083D}">
   <dimension ref="A1:A34"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="6">
         <v>46174</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" s="6">
         <v>46175</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="6">
         <v>46176</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" s="6">
         <v>46177</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" s="6">
         <v>46178</v>
       </c>
     </row>
-    <row r="7" spans="1:1">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" s="6">
         <v>46179</v>
       </c>
     </row>
-    <row r="8" spans="1:1">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" s="6">
         <v>46180</v>
       </c>
     </row>
-    <row r="9" spans="1:1">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" s="6">
         <v>46181</v>
       </c>
     </row>
-    <row r="10" spans="1:1">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" s="6">
         <v>46182</v>
       </c>
     </row>
-    <row r="11" spans="1:1">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" s="6">
         <v>46183</v>
       </c>
     </row>
-    <row r="12" spans="1:1">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" s="6">
         <v>46184</v>
       </c>
     </row>
-    <row r="13" spans="1:1">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" s="6">
         <v>46185</v>
       </c>
     </row>
-    <row r="14" spans="1:1">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" s="6"/>
     </row>
-    <row r="15" spans="1:1">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" s="6"/>
     </row>
-    <row r="16" spans="1:1">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" s="6"/>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" s="6"/>
     </row>
-    <row r="18" spans="1:1">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" s="6"/>
     </row>
-    <row r="19" spans="1:1">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" s="6"/>
     </row>
-    <row r="20" spans="1:1">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" s="6"/>
     </row>
-    <row r="21" spans="1:1">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" s="6"/>
     </row>
-    <row r="22" spans="1:1">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" s="6"/>
     </row>
-    <row r="23" spans="1:1">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" s="6"/>
     </row>
-    <row r="24" spans="1:1">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" s="6"/>
     </row>
-    <row r="25" spans="1:1">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" s="6"/>
     </row>
-    <row r="26" spans="1:1">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" s="6"/>
     </row>
-    <row r="27" spans="1:1">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" s="6"/>
     </row>
-    <row r="28" spans="1:1">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" s="6"/>
     </row>
-    <row r="29" spans="1:1">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" s="6"/>
     </row>
-    <row r="30" spans="1:1">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" s="6"/>
     </row>
-    <row r="31" spans="1:1">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" s="6"/>
     </row>
-    <row r="32" spans="1:1">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" s="6"/>
     </row>
-    <row r="33" spans="1:1">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" s="6"/>
     </row>
-    <row r="34" spans="1:1">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" s="6"/>
     </row>
   </sheetData>
@@ -846,28 +846,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="14.42578125" customWidth="1"/>
-    <col min="3" max="3" width="41.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" customWidth="1"/>
+    <col min="3" max="3" width="41.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.26953125" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="7" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="7" max="8" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.26953125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.1796875" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
-      <c r="B1" s="11" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="B1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-    </row>
-    <row r="2" spans="1:16" ht="30.75">
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+    </row>
+    <row r="2" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
         <v>2</v>
       </c>
@@ -886,17 +886,17 @@
       <c r="F2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="14" t="s">
         <v>8</v>
       </c>
       <c r="H2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -913,14 +913,14 @@
       <c r="F3" s="3">
         <v>9</v>
       </c>
-      <c r="G3" s="16">
+      <c r="G3" s="15">
         <f>E3+F3</f>
         <v>46190</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="14" t="s">
+      <c r="I3" s="13" t="s">
         <v>14</v>
       </c>
       <c r="J3" s="2"/>
@@ -928,7 +928,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -948,21 +948,21 @@
       <c r="F4" s="3">
         <v>18</v>
       </c>
-      <c r="G4" s="16">
+      <c r="G4" s="15">
         <f t="shared" ref="G4:G21" si="0">E4+F4</f>
         <v>46209</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="I4" s="13" t="s">
         <v>14</v>
       </c>
       <c r="P4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -982,21 +982,21 @@
       <c r="F5" s="3">
         <v>7</v>
       </c>
-      <c r="G5" s="16">
+      <c r="G5" s="15">
         <f t="shared" si="0"/>
         <v>46217</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="14" t="s">
+      <c r="I5" s="13" t="s">
         <v>14</v>
       </c>
       <c r="P5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -1016,18 +1016,18 @@
       <c r="F6" s="3">
         <v>2</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="15">
         <f t="shared" si="0"/>
         <v>46220</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16">
+      <c r="I6" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -1047,18 +1047,18 @@
       <c r="F7" s="3">
         <v>7</v>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="15">
         <f t="shared" si="0"/>
         <v>46228</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I7" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16">
+      <c r="I7" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -1078,18 +1078,18 @@
       <c r="F8" s="3">
         <v>7</v>
       </c>
-      <c r="G8" s="16">
+      <c r="G8" s="15">
         <f t="shared" si="0"/>
         <v>46236</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16">
+        <v>17</v>
+      </c>
+      <c r="I8" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -1109,18 +1109,18 @@
       <c r="F9" s="3">
         <v>7</v>
       </c>
-      <c r="G9" s="16">
+      <c r="G9" s="15">
         <f t="shared" si="0"/>
         <v>46244</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I9" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16">
+      <c r="I9" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -1140,18 +1140,18 @@
       <c r="F10" s="3">
         <v>10</v>
       </c>
-      <c r="G10" s="16">
+      <c r="G10" s="15">
         <f t="shared" si="0"/>
         <v>46255</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I10" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16">
+      <c r="I10" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -1171,18 +1171,18 @@
       <c r="F11" s="3">
         <v>7</v>
       </c>
-      <c r="G11" s="16">
+      <c r="G11" s="15">
         <f t="shared" si="0"/>
         <v>46263</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I11" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16">
+      <c r="I11" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -1202,18 +1202,18 @@
       <c r="F12" s="3">
         <v>9</v>
       </c>
-      <c r="G12" s="16">
+      <c r="G12" s="15">
         <f t="shared" si="0"/>
         <v>46273</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I12" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16">
+      <c r="I12" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -1233,18 +1233,18 @@
       <c r="F13" s="3">
         <v>9</v>
       </c>
-      <c r="G13" s="16">
+      <c r="G13" s="15">
         <f t="shared" si="0"/>
         <v>46283</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I13" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16">
+      <c r="I13" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -1264,18 +1264,18 @@
       <c r="F14" s="3">
         <v>5</v>
       </c>
-      <c r="G14" s="16">
+      <c r="G14" s="15">
         <f t="shared" si="0"/>
         <v>46289</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I14" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16">
+      <c r="I14" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -1295,18 +1295,18 @@
       <c r="F15" s="3">
         <v>5</v>
       </c>
-      <c r="G15" s="16">
+      <c r="G15" s="15">
         <f t="shared" si="0"/>
         <v>46295</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I15" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16">
+      <c r="I15" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -1326,18 +1326,18 @@
       <c r="F16" s="3">
         <v>9</v>
       </c>
-      <c r="G16" s="16">
+      <c r="G16" s="15">
         <f t="shared" si="0"/>
         <v>46305</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I16" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
+      <c r="I16" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -1357,18 +1357,18 @@
       <c r="F17" s="3">
         <v>7</v>
       </c>
-      <c r="G17" s="16">
+      <c r="G17" s="15">
         <f t="shared" si="0"/>
         <v>46313</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I17" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
+      <c r="I17" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -1388,18 +1388,18 @@
       <c r="F18" s="3">
         <v>19</v>
       </c>
-      <c r="G18" s="16">
+      <c r="G18" s="15">
         <f t="shared" si="0"/>
         <v>46333</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
+      <c r="I18" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -1419,18 +1419,18 @@
       <c r="F19" s="3">
         <v>9</v>
       </c>
-      <c r="G19" s="16">
+      <c r="G19" s="15">
         <f t="shared" si="0"/>
         <v>46343</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I19" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
+      <c r="I19" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -1450,18 +1450,18 @@
       <c r="F20" s="3">
         <v>9</v>
       </c>
-      <c r="G20" s="16">
+      <c r="G20" s="15">
         <f t="shared" si="0"/>
         <v>46353</v>
       </c>
       <c r="H20" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I20" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
+      <c r="I20" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -1481,22 +1481,22 @@
       <c r="F21" s="3">
         <v>9</v>
       </c>
-      <c r="G21" s="16">
+      <c r="G21" s="15">
         <f t="shared" si="0"/>
         <v>46363</v>
       </c>
       <c r="H21" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I21" s="14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="15">
+      <c r="I21" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="C23" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="11">
         <f>G21</f>
         <v>46363</v>
       </c>
@@ -1523,9 +1523,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBB1C660-FD22-424D-B761-DA960EAAB43D}">
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -1551,7 +1551,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1571,7 +1571,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1588,7 +1588,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1605,7 +1605,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1622,7 +1622,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1639,7 +1639,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1656,7 +1656,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1673,7 +1673,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
updated some code in employee module
</commit_message>
<xml_diff>
--- a/DWM.xlsx
+++ b/DWM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bnagritech1-my.sharepoint.com/personal/it_intern_bngroupindia_com/Documents/tradesphere/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="492" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC48B3EA-9294-42A7-91D6-A116C54D00DA}"/>
+  <xr:revisionPtr revIDLastSave="495" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8EED81F-56EE-4182-8445-F9C94655C3C6}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="1140" yWindow="1140" windowWidth="14400" windowHeight="7270" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="73">
   <si>
     <t>Pilot : Tradesphere</t>
   </si>
@@ -395,10 +395,10 @@
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -722,256 +722,262 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="16">
+      <c r="A2" s="8">
         <v>46174</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" s="16">
+      <c r="A3" s="8">
         <v>46175</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" s="16">
+      <c r="A4" s="8">
         <v>46176</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" s="16">
+      <c r="A5" s="8">
         <v>46177</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" s="16">
+      <c r="A6" s="8">
         <v>46178</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" s="16">
+      <c r="A7" s="8">
         <v>46179</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="16">
+      <c r="A8" s="8">
         <v>46180</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" s="16">
+      <c r="A9" s="8">
         <v>46181</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" s="16">
+      <c r="A10" s="8">
         <v>46182</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="16">
+      <c r="A11" s="8">
         <v>46183</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" s="16">
+      <c r="A12" s="8">
         <v>46184</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" s="16">
+      <c r="A13" s="8">
         <v>46185</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" s="16">
+      <c r="A14" s="8">
         <v>46186</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" s="16">
+      <c r="A15" s="8">
         <v>46187</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" s="16">
+      <c r="A16" s="8">
         <v>46188</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:2">
-      <c r="A17" s="16">
+      <c r="A17" s="8">
         <v>46189</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:2">
-      <c r="A18" s="16">
+      <c r="A18" s="8">
         <v>46190</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:2">
-      <c r="A19" s="16">
+      <c r="A19" s="8">
         <v>46191</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:2">
-      <c r="A20" s="16">
+      <c r="A20" s="8">
         <v>46192</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:2">
-      <c r="A21" s="16">
+      <c r="A21" s="8">
         <v>46193</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:2">
-      <c r="A22" s="16">
+      <c r="A22" s="8">
         <v>46194</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2">
-      <c r="A23" s="16">
+      <c r="A23" s="8">
         <v>46195</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:2">
-      <c r="A24" s="16">
+      <c r="A24" s="8">
         <v>46196</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:2">
-      <c r="A25" s="16">
+      <c r="A25" s="8">
         <v>46197</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:2">
-      <c r="A26" s="16">
+      <c r="A26" s="8">
         <v>46198</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:2">
-      <c r="A27" s="16">
+      <c r="A27" s="8">
         <v>46199</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:2">
-      <c r="A28" s="16">
+      <c r="A28" s="8">
         <v>46200</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:2">
-      <c r="A29" s="16">
+      <c r="A29" s="8">
         <v>46201</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:2">
-      <c r="A30" s="16">
+      <c r="A30" s="8">
         <v>46202</v>
       </c>
+      <c r="B30" s="3" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="31" spans="1:2">
-      <c r="A31" s="16">
+      <c r="A31" s="8">
         <v>46203</v>
       </c>
+      <c r="B31" s="3" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="32" spans="1:2">
-      <c r="A32" s="16">
+      <c r="A32" s="15">
         <v>46204</v>
       </c>
     </row>
     <row r="33" spans="1:2">
-      <c r="A33" s="16">
+      <c r="A33" s="15">
         <v>46205</v>
       </c>
     </row>
     <row r="34" spans="1:2">
-      <c r="A34" s="16">
+      <c r="A34" s="15">
         <v>46206</v>
       </c>
     </row>
     <row r="35" spans="1:2">
-      <c r="A35" s="16">
+      <c r="A35" s="15">
         <v>46207</v>
       </c>
       <c r="B35" t="s">
@@ -979,7 +985,7 @@
       </c>
     </row>
     <row r="36" spans="1:2">
-      <c r="A36" s="16">
+      <c r="A36" s="15">
         <v>46208</v>
       </c>
       <c r="B36" t="s">
@@ -987,77 +993,77 @@
       </c>
     </row>
     <row r="37" spans="1:2">
-      <c r="A37" s="16">
+      <c r="A37" s="15">
         <v>46209</v>
       </c>
     </row>
     <row r="38" spans="1:2">
-      <c r="A38" s="16">
+      <c r="A38" s="15">
         <v>46210</v>
       </c>
     </row>
     <row r="39" spans="1:2">
-      <c r="A39" s="16">
+      <c r="A39" s="15">
         <v>46211</v>
       </c>
     </row>
     <row r="40" spans="1:2">
-      <c r="A40" s="16">
+      <c r="A40" s="15">
         <v>46212</v>
       </c>
     </row>
     <row r="41" spans="1:2">
-      <c r="A41" s="16">
+      <c r="A41" s="15">
         <v>46213</v>
       </c>
     </row>
     <row r="42" spans="1:2">
-      <c r="A42" s="16">
+      <c r="A42" s="15">
         <v>46214</v>
       </c>
     </row>
     <row r="43" spans="1:2">
-      <c r="A43" s="16">
+      <c r="A43" s="15">
         <v>46215</v>
       </c>
     </row>
     <row r="44" spans="1:2">
-      <c r="A44" s="16">
+      <c r="A44" s="15">
         <v>46216</v>
       </c>
     </row>
     <row r="45" spans="1:2">
-      <c r="A45" s="16">
+      <c r="A45" s="15">
         <v>46217</v>
       </c>
     </row>
     <row r="46" spans="1:2">
-      <c r="A46" s="16">
+      <c r="A46" s="15">
         <v>46218</v>
       </c>
     </row>
     <row r="47" spans="1:2">
-      <c r="A47" s="16">
+      <c r="A47" s="15">
         <v>46219</v>
       </c>
     </row>
     <row r="48" spans="1:2">
-      <c r="A48" s="16">
+      <c r="A48" s="15">
         <v>46220</v>
       </c>
     </row>
     <row r="49" spans="1:1">
-      <c r="A49" s="16">
+      <c r="A49" s="15">
         <v>46221</v>
       </c>
     </row>
     <row r="50" spans="1:1">
-      <c r="A50" s="16">
+      <c r="A50" s="15">
         <v>46222</v>
       </c>
     </row>
     <row r="51" spans="1:1">
-      <c r="A51" s="16">
+      <c r="A51" s="15">
         <v>46223</v>
       </c>
     </row>
@@ -1082,13 +1088,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" spans="1:16" ht="29.1">
       <c r="A2" s="6" t="s">

</xml_diff>

<commit_message>
added abstract method in RetailerRepository.java
</commit_message>
<xml_diff>
--- a/DWM.xlsx
+++ b/DWM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bnagritech1-my.sharepoint.com/personal/it_intern_bngroupindia_com/Documents/tradesphere/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="507" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76BAE026-BEC1-414A-904B-7D15A3B575C5}"/>
+  <xr:revisionPtr revIDLastSave="508" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB553083-A726-404D-B66F-044C0151ED47}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1140" yWindow="1140" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DWM" sheetId="4" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="73">
   <si>
     <t>Pilot : Tradesphere</t>
   </si>
@@ -1026,7 +1026,9 @@
       <c r="A37" s="8">
         <v>46209</v>
       </c>
-      <c r="B37" s="3"/>
+      <c r="B37" s="3" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" s="8">

</xml_diff>

<commit_message>
created RetailerController.java in controller
</commit_message>
<xml_diff>
--- a/DWM.xlsx
+++ b/DWM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bnagritech1-my.sharepoint.com/personal/it_intern_bngroupindia_com/Documents/tradesphere/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="508" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB553083-A726-404D-B66F-044C0151ED47}"/>
+  <xr:revisionPtr revIDLastSave="509" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C447CF16-F258-41AB-ABC4-BA918A05DAA4}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="1140" yWindow="1140" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="73">
   <si>
     <t>Pilot : Tradesphere</t>
   </si>
@@ -1034,7 +1034,9 @@
       <c r="A38" s="8">
         <v>46210</v>
       </c>
-      <c r="B38" s="3"/>
+      <c r="B38" s="3" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" s="8">

</xml_diff>

<commit_message>
added some fields in user.java and created ForgotPasswordRequest.java
</commit_message>
<xml_diff>
--- a/DWM.xlsx
+++ b/DWM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bnagritech1-my.sharepoint.com/personal/it_intern_bngroupindia_com/Documents/tradesphere/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="509" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C447CF16-F258-41AB-ABC4-BA918A05DAA4}"/>
+  <xr:revisionPtr revIDLastSave="511" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50AC04F1-B4E1-47B9-8C0F-E46B050BDCF0}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1140" yWindow="1140" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DWM" sheetId="4" r:id="rId1"/>
@@ -1454,7 +1454,7 @@
         <v>46230</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="I9" s="12" t="s">
         <v>16</v>
@@ -1485,7 +1485,7 @@
         <v>46236</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="I10" s="12" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
created Beat.java and BeatRetailer.java and added fields in it
</commit_message>
<xml_diff>
--- a/DWM.xlsx
+++ b/DWM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bnagritech1-my.sharepoint.com/personal/it_intern_bngroupindia_com/Documents/tradesphere/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="513" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57B82C4A-3268-4283-A25D-655CC3EA2828}"/>
+  <xr:revisionPtr revIDLastSave="514" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{480EE0AB-2328-4D42-88C2-D33718E53118}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1140" yWindow="1140" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DWM" sheetId="4" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="73">
   <si>
     <t>Pilot : Tradesphere</t>
   </si>
@@ -1058,7 +1058,9 @@
       <c r="A41" s="8">
         <v>46213</v>
       </c>
-      <c r="B41" s="3"/>
+      <c r="B41" s="3" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" s="8">

</xml_diff>

<commit_message>
added addProduct method EmployeeController.java
</commit_message>
<xml_diff>
--- a/DWM.xlsx
+++ b/DWM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bnagritech1-my.sharepoint.com/personal/it_intern_bngroupindia_com/Documents/tradesphere/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="543" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33B5B534-AD42-44FF-A243-F930FA05171C}"/>
+  <xr:revisionPtr revIDLastSave="545" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C7FCA8B-8E18-4F05-8FF9-95B1F29BF057}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1140" yWindow="1140" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DWM" sheetId="4" r:id="rId1"/>
@@ -273,7 +273,7 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
     <numFmt numFmtId="165" formatCode="[$-409]dd\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -746,17 +746,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A0EB679-3C26-4760-A69A-4B3B2033083D}">
   <dimension ref="A1:B60"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="8">
         <v>46174</v>
       </c>
@@ -764,7 +764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="8">
         <v>46175</v>
       </c>
@@ -772,7 +772,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="8">
         <v>46176</v>
       </c>
@@ -780,7 +780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="8">
         <v>46177</v>
       </c>
@@ -788,7 +788,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="8">
         <v>46178</v>
       </c>
@@ -796,7 +796,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="8">
         <v>46179</v>
       </c>
@@ -804,7 +804,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="8">
         <v>46180</v>
       </c>
@@ -812,7 +812,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="8">
         <v>46181</v>
       </c>
@@ -820,7 +820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="8">
         <v>46182</v>
       </c>
@@ -828,7 +828,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="8">
         <v>46183</v>
       </c>
@@ -836,7 +836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="8">
         <v>46184</v>
       </c>
@@ -844,7 +844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="8">
         <v>46185</v>
       </c>
@@ -852,7 +852,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="8">
         <v>46186</v>
       </c>
@@ -860,7 +860,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="8">
         <v>46187</v>
       </c>
@@ -868,7 +868,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="8">
         <v>46188</v>
       </c>
@@ -876,7 +876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="8">
         <v>46189</v>
       </c>
@@ -884,7 +884,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="8">
         <v>46190</v>
       </c>
@@ -892,7 +892,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="8">
         <v>46191</v>
       </c>
@@ -900,7 +900,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="8">
         <v>46192</v>
       </c>
@@ -908,7 +908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="8">
         <v>46193</v>
       </c>
@@ -916,7 +916,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="8">
         <v>46194</v>
       </c>
@@ -924,7 +924,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" s="8">
         <v>46195</v>
       </c>
@@ -932,7 +932,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="8">
         <v>46196</v>
       </c>
@@ -940,7 +940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="8">
         <v>46197</v>
       </c>
@@ -948,7 +948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="8">
         <v>46198</v>
       </c>
@@ -956,7 +956,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="8">
         <v>46199</v>
       </c>
@@ -964,7 +964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="8">
         <v>46200</v>
       </c>
@@ -972,7 +972,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" s="8">
         <v>46201</v>
       </c>
@@ -980,7 +980,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="8">
         <v>46202</v>
       </c>
@@ -988,7 +988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" s="15">
         <v>46203</v>
       </c>
@@ -996,7 +996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="8">
         <v>46204</v>
       </c>
@@ -1004,7 +1004,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" s="8">
         <v>46205</v>
       </c>
@@ -1012,7 +1012,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" s="8">
         <v>46206</v>
       </c>
@@ -1020,7 +1020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" s="8">
         <v>46207</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" s="8">
         <v>46208</v>
       </c>
@@ -1036,7 +1036,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" s="8">
         <v>46209</v>
       </c>
@@ -1044,7 +1044,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" s="8">
         <v>46210</v>
       </c>
@@ -1052,7 +1052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" s="8">
         <v>46211</v>
       </c>
@@ -1060,7 +1060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" s="8">
         <v>46212</v>
       </c>
@@ -1068,7 +1068,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" s="8">
         <v>46213</v>
       </c>
@@ -1076,7 +1076,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" s="8">
         <v>46214</v>
       </c>
@@ -1084,7 +1084,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" s="8">
         <v>46215</v>
       </c>
@@ -1092,7 +1092,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" s="8">
         <v>46216</v>
       </c>
@@ -1100,7 +1100,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" s="8">
         <v>46217</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" s="8">
         <v>46218</v>
       </c>
@@ -1116,7 +1116,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" s="8">
         <v>46219</v>
       </c>
@@ -1124,7 +1124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" s="8">
         <v>46220</v>
       </c>
@@ -1132,7 +1132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" s="8">
         <v>46221</v>
       </c>
@@ -1140,7 +1140,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:2">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" s="8">
         <v>46222</v>
       </c>
@@ -1148,7 +1148,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" s="8">
         <v>46223</v>
       </c>
@@ -1156,33 +1156,33 @@
         <v>4</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" s="8">
         <v>46224</v>
       </c>
-      <c r="B52" s="3"/>
-    </row>
-    <row r="53" spans="1:2">
+      <c r="B52" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" s="8">
         <v>46225</v>
       </c>
       <c r="B53" s="3"/>
     </row>
-    <row r="54" spans="1:2">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" s="8">
         <v>46226</v>
       </c>
       <c r="B54" s="3"/>
     </row>
-    <row r="55" spans="1:2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" s="8">
         <v>46227</v>
       </c>
-      <c r="B55" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2">
+      <c r="B55" s="3"/>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" s="8">
         <v>46228</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="1:2">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" s="8">
         <v>46229</v>
       </c>
@@ -1198,19 +1198,19 @@
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="1:2">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" s="8">
         <v>46230</v>
       </c>
       <c r="B58" s="3"/>
     </row>
-    <row r="59" spans="1:2">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" s="8">
         <v>46231</v>
       </c>
       <c r="B59" s="3"/>
     </row>
-    <row r="60" spans="1:2">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" s="8">
         <v>46232</v>
       </c>
@@ -1232,19 +1232,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P23"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="14.42578125" customWidth="1"/>
-    <col min="3" max="3" width="38.140625" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" customWidth="1"/>
+    <col min="3" max="3" width="38.1796875" customWidth="1"/>
+    <col min="4" max="4" width="13.26953125" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="7" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" hidden="1" customWidth="1"/>
+    <col min="7" max="8" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.26953125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.1796875" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="B1" s="18" t="s">
         <v>5</v>
       </c>
@@ -1253,7 +1253,7 @@
       <c r="E1" s="18"/>
       <c r="F1" s="18"/>
     </row>
-    <row r="2" spans="1:16" ht="29.1">
+    <row r="2" spans="1:16" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>6</v>
       </c>
@@ -1282,7 +1282,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -1348,7 +1348,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -1382,7 +1382,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -1413,7 +1413,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -1444,7 +1444,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:16">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -1475,7 +1475,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -1506,7 +1506,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -1537,7 +1537,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:16">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -1568,7 +1568,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:16">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -1599,7 +1599,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:16">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:16">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -1661,7 +1661,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:16">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -1692,7 +1692,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:16">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -1723,7 +1723,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -1754,7 +1754,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -1788,7 +1788,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -1819,7 +1819,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -1850,7 +1850,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="C23" s="3" t="s">
         <v>58</v>
       </c>
@@ -1912,9 +1912,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBB1C660-FD22-424D-B761-DA960EAAB43D}">
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>6</v>
       </c>
@@ -1940,7 +1940,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1960,7 +1960,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1977,7 +1977,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1994,7 +1994,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2011,7 +2011,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2028,7 +2028,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2045,7 +2045,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2062,7 +2062,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
created Order.java class in order module
</commit_message>
<xml_diff>
--- a/DWM.xlsx
+++ b/DWM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bnagritech1-my.sharepoint.com/personal/it_intern_bngroupindia_com/Documents/tradesphere/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bnagritech1-my.sharepoint.com/personal/mohini_chaturvedi_bngroupindia_com/Documents/tradesphere/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="564" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{165980CE-C56C-4AAD-BD8D-2682C91F4E10}"/>
+  <xr:revisionPtr revIDLastSave="566" documentId="11_F25DC773A252ABDACC1048B9199B6F7E5ADE58EA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9763CD56-BEA7-4361-B970-84D0B99D0101}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="76">
   <si>
     <t>Pilot : Tradesphere</t>
   </si>
@@ -263,6 +263,9 @@
   </si>
   <si>
     <t>App will be developed after the final submission and testing.</t>
+  </si>
+  <si>
+    <t>merge with order module</t>
   </si>
 </sst>
 </file>
@@ -1654,7 +1657,7 @@
         <v>46257</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>24</v>
+        <v>75</v>
       </c>
       <c r="I13" s="12" t="s">
         <v>18</v>
@@ -1747,7 +1750,7 @@
         <v>46283</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I16" s="12" t="s">
         <v>18</v>

</xml_diff>